<commit_message>
solves SISOR download via DPM install - issue 41
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_QDD_PLURIANUAL_INVEST.xlsx
+++ b/bancos/SISOR/BASE_QDD_PLURIANUAL_INVEST.xlsx
@@ -1,43 +1,288 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <workbookPr date1904="false"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BASE_QDD_PLURIANUAL_INVEST" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="BASE_QDD_PLURIANUAL_INVEST" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="82">
+  <si>
+    <t xml:space="preserve">ANO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COD_ORGAO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DESC_ORGAO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COD_UO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DESC_UO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FUNCAO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUBFUNCAO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COD_PROGRAMA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDENT_PROJATIV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROJ_ATIV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AÇÃO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUBPROJETO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CATEGORIA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FONTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IAG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROGRAMA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACAO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VALOR (R$) 2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VALOR (R$) 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VALOR (R$) 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VALOR (R$) 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMPANHIA DE DESENVOLVIMENTO ECONÔMICO DE MINAS GERAIS - CODEMIG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MINAS GERAÇÃO DE VALOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MANUTENÇÃO E AQUISIÇÕES DA CODEMIG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMPANHIA DE DESENVOLVIMENTO DE MINAS GERAIS - CODEMG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GESTÃO DE INFRAESTRUTURA, CONSÓRCIOS E EQUIPAMENTOS CULTURAIS E TURÍSTICOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMPANHIA DE HABITAÇÃO DO ESTADO DE MINAS GERAIS - COHAB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">APOIO ÀS POLÍTICAS PÚBLICAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA - COHAB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMPANHIA DE SANEAMENTO DE MINAS GERAIS  - COPASA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SANEAMENTO E RESÍDUOS ESPECIAIS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PPP SISTEMA ADUTOR RIO MANSO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMPANHIA ENERGÉTICA DE MINAS GERAIS - CEMIG HOLDING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INVESTIMENTOS CEMIG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AGÊNCIA DE PROMOÇÃO DE INVESTIMENTOS DE MINAS GERAIS - INVEST MINAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL - INDI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DESENVOLVIMENTO SOCIOECONÔMICO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INVESTIMENTO NA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL  DO BDMG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMPANHIA DE GÁS DE MINAS GERAIS - GASMIG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GERAÇÃO DE ENERGIA ELÉTRICA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG GERAÇÃO E TRANSMISSÃO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SECRETARIA DE ESTADO DE INFRAESTRUTURA, MOBILIDADE E PARCERIA - SEINFRA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TREM METROPOLITANO DE BELO HORIZONTE S.A - TREM METROPOLITANO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOLUÇÕES EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,94 +290,17 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <dxfs count="0"/>
 </styleSheet>
 </file>
 
@@ -182,10 +350,6 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -211,15 +375,12 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -245,6 +406,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -420,140 +582,90 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:U41"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>ANO</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>COD_ORGAO</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>DESC_ORGAO</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>COD_UO</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>DESC_UO</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>FUNCAO</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>SUBFUNCAO</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>COD_PROGRAMA</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>IDENT_PROJATIV</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>PROJ_ATIV</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>AÇÃO</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>SUBPROJETO</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>CATEGORIA</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>FONTE</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>IAG</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>PROGRAMA</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>ACAO</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>VALOR (R$) 2024</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>VALOR (R$) 2025</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>VALOR (R$) 2026</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>VALOR (R$) 2027</t>
-        </is>
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="n">
         <v>2024</v>
       </c>
       <c r="B2" t="n">
         <v>1220</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C2" t="s">
+        <v>21</v>
       </c>
       <c r="D2" t="n">
         <v>5011</v>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>COMPANHIA DE DESENVOLVIMENTO ECONÔMICO DE MINAS GERAIS - CODEMIG</t>
-        </is>
+      <c r="E2" t="s">
+        <v>22</v>
       </c>
       <c r="F2" t="n">
         <v>4</v>
@@ -585,15 +697,11 @@
       <c r="O2" t="n">
         <v>0</v>
       </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>MINAS GERAÇÃO DE VALOR</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>MANUTENÇÃO E AQUISIÇÕES DA CODEMIG</t>
-        </is>
+      <c r="P2" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>24</v>
       </c>
       <c r="R2" t="n">
         <v>1000</v>
@@ -609,24 +717,20 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="n">
         <v>2024</v>
       </c>
       <c r="B3" t="n">
         <v>1220</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C3" t="s">
+        <v>21</v>
       </c>
       <c r="D3" t="n">
         <v>5031</v>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>COMPANHIA DE DESENVOLVIMENTO DE MINAS GERAIS - CODEMG</t>
-        </is>
+      <c r="E3" t="s">
+        <v>25</v>
       </c>
       <c r="F3" t="n">
         <v>19</v>
@@ -658,15 +762,11 @@
       <c r="O3" t="n">
         <v>0</v>
       </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>MINAS GERAÇÃO DE VALOR</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>GESTÃO DE INFRAESTRUTURA, CONSÓRCIOS E EQUIPAMENTOS CULTURAIS E TURÍSTICOS</t>
-        </is>
+      <c r="P3" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>26</v>
       </c>
       <c r="R3" t="n">
         <v>12580000</v>
@@ -682,24 +782,20 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="n">
         <v>2024</v>
       </c>
       <c r="B4" t="n">
         <v>1220</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C4" t="s">
+        <v>21</v>
       </c>
       <c r="D4" t="n">
         <v>5071</v>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>COMPANHIA DE HABITAÇÃO DO ESTADO DE MINAS GERAIS - COHAB</t>
-        </is>
+      <c r="E4" t="s">
+        <v>27</v>
       </c>
       <c r="F4" t="n">
         <v>16</v>
@@ -731,15 +827,11 @@
       <c r="O4" t="n">
         <v>0</v>
       </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA - COHAB</t>
-        </is>
+      <c r="P4" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>29</v>
       </c>
       <c r="R4" t="n">
         <v>120000</v>
@@ -755,24 +847,20 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" t="n">
         <v>2024</v>
       </c>
       <c r="B5" t="n">
         <v>1220</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C5" t="s">
+        <v>21</v>
       </c>
       <c r="D5" t="n">
         <v>5081</v>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
-        </is>
+      <c r="E5" t="s">
+        <v>30</v>
       </c>
       <c r="F5" t="n">
         <v>17</v>
@@ -804,15 +892,11 @@
       <c r="O5" t="n">
         <v>0</v>
       </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
-        </is>
+      <c r="P5" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>32</v>
       </c>
       <c r="R5" t="n">
         <v>50000000</v>
@@ -828,24 +912,20 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" t="n">
         <v>2024</v>
       </c>
       <c r="B6" t="n">
         <v>1220</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C6" t="s">
+        <v>21</v>
       </c>
       <c r="D6" t="n">
         <v>5081</v>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
-        </is>
+      <c r="E6" t="s">
+        <v>30</v>
       </c>
       <c r="F6" t="n">
         <v>17</v>
@@ -877,15 +957,11 @@
       <c r="O6" t="n">
         <v>0</v>
       </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - COPASA</t>
-        </is>
+      <c r="P6" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>32</v>
       </c>
       <c r="R6" t="n">
         <v>50000000</v>
@@ -901,24 +977,20 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" t="n">
         <v>2024</v>
       </c>
       <c r="B7" t="n">
         <v>1220</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C7" t="s">
+        <v>21</v>
       </c>
       <c r="D7" t="n">
         <v>5081</v>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
-        </is>
+      <c r="E7" t="s">
+        <v>30</v>
       </c>
       <c r="F7" t="n">
         <v>17</v>
@@ -950,15 +1022,11 @@
       <c r="O7" t="n">
         <v>0</v>
       </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
-        </is>
+      <c r="P7" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>33</v>
       </c>
       <c r="R7" t="n">
         <v>250000000</v>
@@ -974,24 +1042,20 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" t="n">
         <v>2024</v>
       </c>
       <c r="B8" t="n">
         <v>1220</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C8" t="s">
+        <v>21</v>
       </c>
       <c r="D8" t="n">
         <v>5081</v>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
-        </is>
+      <c r="E8" t="s">
+        <v>30</v>
       </c>
       <c r="F8" t="n">
         <v>17</v>
@@ -1023,15 +1087,11 @@
       <c r="O8" t="n">
         <v>0</v>
       </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
-        </is>
+      <c r="P8" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>33</v>
       </c>
       <c r="R8" t="n">
         <v>1062500000</v>
@@ -1047,24 +1107,20 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" t="n">
         <v>2024</v>
       </c>
       <c r="B9" t="n">
         <v>1220</v>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C9" t="s">
+        <v>21</v>
       </c>
       <c r="D9" t="n">
         <v>5081</v>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
-        </is>
+      <c r="E9" t="s">
+        <v>30</v>
       </c>
       <c r="F9" t="n">
         <v>17</v>
@@ -1096,15 +1152,11 @@
       <c r="O9" t="n">
         <v>0</v>
       </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
-        </is>
+      <c r="P9" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>33</v>
       </c>
       <c r="R9" t="n">
         <v>40000000</v>
@@ -1120,24 +1172,20 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" t="n">
         <v>2024</v>
       </c>
       <c r="B10" t="n">
         <v>1220</v>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C10" t="s">
+        <v>21</v>
       </c>
       <c r="D10" t="n">
         <v>5081</v>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
-        </is>
+      <c r="E10" t="s">
+        <v>30</v>
       </c>
       <c r="F10" t="n">
         <v>17</v>
@@ -1169,15 +1217,11 @@
       <c r="O10" t="n">
         <v>0</v>
       </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
-        </is>
+      <c r="P10" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>33</v>
       </c>
       <c r="R10" t="n">
         <v>100000000</v>
@@ -1193,24 +1237,20 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" t="n">
         <v>2024</v>
       </c>
       <c r="B11" t="n">
         <v>1220</v>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C11" t="s">
+        <v>21</v>
       </c>
       <c r="D11" t="n">
         <v>5081</v>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
-        </is>
+      <c r="E11" t="s">
+        <v>30</v>
       </c>
       <c r="F11" t="n">
         <v>17</v>
@@ -1242,15 +1282,11 @@
       <c r="O11" t="n">
         <v>0</v>
       </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DA COPASA</t>
-        </is>
+      <c r="P11" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>33</v>
       </c>
       <c r="R11" t="n">
         <v>97500000</v>
@@ -1266,24 +1302,20 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" t="n">
         <v>2024</v>
       </c>
       <c r="B12" t="n">
         <v>1220</v>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C12" t="s">
+        <v>21</v>
       </c>
       <c r="D12" t="n">
         <v>5081</v>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>COMPANHIA DE SANEAMENTO DE MINAS GERAIS - COPASA</t>
-        </is>
+      <c r="E12" t="s">
+        <v>30</v>
       </c>
       <c r="F12" t="n">
         <v>17</v>
@@ -1315,15 +1347,11 @@
       <c r="O12" t="n">
         <v>0</v>
       </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>PPP SISTEMA ADUTOR RIO MANSO</t>
-        </is>
+      <c r="P12" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>34</v>
       </c>
       <c r="R12" t="n">
         <v>45752420</v>
@@ -1339,24 +1367,20 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" t="n">
         <v>2024</v>
       </c>
       <c r="B13" t="n">
         <v>1220</v>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C13" t="s">
+        <v>21</v>
       </c>
       <c r="D13" t="n">
         <v>5121</v>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>COMPANHIA ENERGÉTICA DE MINAS GERAIS - CEMIG HOLDING</t>
-        </is>
+      <c r="E13" t="s">
+        <v>35</v>
       </c>
       <c r="F13" t="n">
         <v>25</v>
@@ -1388,15 +1412,11 @@
       <c r="O13" t="n">
         <v>0</v>
       </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>INVESTIMENTOS CEMIG</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG HOLDING</t>
-        </is>
+      <c r="P13" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>37</v>
       </c>
       <c r="R13" t="n">
         <v>344720630</v>
@@ -1412,24 +1432,20 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" t="n">
         <v>2024</v>
       </c>
       <c r="B14" t="n">
         <v>1220</v>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C14" t="s">
+        <v>21</v>
       </c>
       <c r="D14" t="n">
         <v>5121</v>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>COMPANHIA ENERGÉTICA DE MINAS GERAIS - CEMIG HOLDING</t>
-        </is>
+      <c r="E14" t="s">
+        <v>35</v>
       </c>
       <c r="F14" t="n">
         <v>25</v>
@@ -1461,15 +1477,11 @@
       <c r="O14" t="n">
         <v>0</v>
       </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>INVESTIMENTOS CEMIG</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA CEMIG HOLDING</t>
-        </is>
+      <c r="P14" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>38</v>
       </c>
       <c r="R14" t="n">
         <v>40000</v>
@@ -1485,24 +1497,20 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" t="n">
         <v>2024</v>
       </c>
       <c r="B15" t="n">
         <v>1220</v>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C15" t="s">
+        <v>21</v>
       </c>
       <c r="D15" t="n">
         <v>5131</v>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>AGÊNCIA DE PROMOÇÃO DE INVESTIMENTOS DE MINAS GERAIS - INVEST MINAS</t>
-        </is>
+      <c r="E15" t="s">
+        <v>39</v>
       </c>
       <c r="F15" t="n">
         <v>22</v>
@@ -1534,15 +1542,11 @@
       <c r="O15" t="n">
         <v>0</v>
       </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL - INDI</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
-        <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
-        </is>
+      <c r="P15" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>41</v>
       </c>
       <c r="R15" t="n">
         <v>500000</v>
@@ -1558,24 +1562,20 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" t="n">
         <v>2024</v>
       </c>
       <c r="B16" t="n">
         <v>1220</v>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C16" t="s">
+        <v>21</v>
       </c>
       <c r="D16" t="n">
         <v>5131</v>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>AGÊNCIA DE PROMOÇÃO DE INVESTIMENTOS DE MINAS GERAIS - INVEST MINAS</t>
-        </is>
+      <c r="E16" t="s">
+        <v>39</v>
       </c>
       <c r="F16" t="n">
         <v>22</v>
@@ -1607,15 +1607,11 @@
       <c r="O16" t="n">
         <v>0</v>
       </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL - INDI</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA INVEST MINAS</t>
-        </is>
+      <c r="P16" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>41</v>
       </c>
       <c r="R16" t="n">
         <v>0</v>
@@ -1631,24 +1627,20 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" t="n">
         <v>2024</v>
       </c>
       <c r="B17" t="n">
         <v>1220</v>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C17" t="s">
+        <v>21</v>
       </c>
       <c r="D17" t="n">
         <v>5191</v>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
-        </is>
+      <c r="E17" t="s">
+        <v>42</v>
       </c>
       <c r="F17" t="n">
         <v>4</v>
@@ -1680,15 +1672,11 @@
       <c r="O17" t="n">
         <v>0</v>
       </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
-        <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRAESTRUTURA DA MGI</t>
-        </is>
+      <c r="P17" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>44</v>
       </c>
       <c r="R17" t="n">
         <v>670000</v>
@@ -1704,24 +1692,20 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" t="n">
         <v>2024</v>
       </c>
       <c r="B18" t="n">
         <v>1220</v>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C18" t="s">
+        <v>21</v>
       </c>
       <c r="D18" t="n">
         <v>5191</v>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
-        </is>
+      <c r="E18" t="s">
+        <v>42</v>
       </c>
       <c r="F18" t="n">
         <v>4</v>
@@ -1753,15 +1737,11 @@
       <c r="O18" t="n">
         <v>0</v>
       </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>DESENVOLVIMENTO SOCIOECONÔMICO</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
-        </is>
+      <c r="P18" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>46</v>
       </c>
       <c r="R18" t="n">
         <v>1000</v>
@@ -1777,24 +1757,20 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" t="n">
         <v>2024</v>
       </c>
       <c r="B19" t="n">
         <v>1220</v>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C19" t="s">
+        <v>21</v>
       </c>
       <c r="D19" t="n">
         <v>5191</v>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
-        </is>
+      <c r="E19" t="s">
+        <v>42</v>
       </c>
       <c r="F19" t="n">
         <v>4</v>
@@ -1826,15 +1802,11 @@
       <c r="O19" t="n">
         <v>0</v>
       </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>DESENVOLVIMENTO SOCIOECONÔMICO</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>SUPORTE AO DESENVOLVIMENTO ESTADUAL</t>
-        </is>
+      <c r="P19" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>46</v>
       </c>
       <c r="R19" t="n">
         <v>186000</v>
@@ -1850,24 +1822,20 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" t="n">
         <v>2024</v>
       </c>
       <c r="B20" t="n">
         <v>1220</v>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C20" t="s">
+        <v>21</v>
       </c>
       <c r="D20" t="n">
         <v>5191</v>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>MINAS GERAIS PARTICIPAÇÕES S.A - MGI</t>
-        </is>
+      <c r="E20" t="s">
+        <v>42</v>
       </c>
       <c r="F20" t="n">
         <v>4</v>
@@ -1899,15 +1867,11 @@
       <c r="O20" t="n">
         <v>0</v>
       </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>APORTE DE CAPITAL E MANUTENÇÃO DA INFRAESTRUTURA DA MGI</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>INVESTIMENTOS VIA PARTICIPAÇÃO SOCIETÁRIA</t>
-        </is>
+      <c r="P20" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>47</v>
       </c>
       <c r="R20" t="n">
         <v>1000</v>
@@ -1923,24 +1887,20 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" t="n">
         <v>2024</v>
       </c>
       <c r="B21" t="n">
         <v>1220</v>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C21" t="s">
+        <v>21</v>
       </c>
       <c r="D21" t="n">
         <v>5201</v>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
-        </is>
+      <c r="E21" t="s">
+        <v>48</v>
       </c>
       <c r="F21" t="n">
         <v>23</v>
@@ -1972,15 +1932,11 @@
       <c r="O21" t="n">
         <v>0</v>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>INVESTIMENTO NA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL DO BDMG</t>
-        </is>
+      <c r="P21" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>50</v>
       </c>
       <c r="R21" t="n">
         <v>23908160</v>
@@ -1996,24 +1952,20 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" t="n">
         <v>2024</v>
       </c>
       <c r="B22" t="n">
         <v>1220</v>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C22" t="s">
+        <v>21</v>
       </c>
       <c r="D22" t="n">
         <v>5201</v>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>BANCO DE DESENVOLVIMENTO DE MINAS GERAIS S.A - BDMG</t>
-        </is>
+      <c r="E22" t="s">
+        <v>48</v>
       </c>
       <c r="F22" t="n">
         <v>23</v>
@@ -2045,15 +1997,11 @@
       <c r="O22" t="n">
         <v>0</v>
       </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
-        </is>
-      </c>
-      <c r="Q22" t="inlineStr">
-        <is>
-          <t>FINANCIAMENTO À INFRAESTRUTURA E AO DESENVOLVIMENTO SUSTENTÁVEL EM MG ENTRE BDMG E NEW DEVELOPMENT BANK (BDMG INFRA ODS)</t>
-        </is>
+      <c r="P22" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>51</v>
       </c>
       <c r="R22" t="n">
         <v>600000000</v>
@@ -2069,24 +2017,20 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" t="n">
         <v>2024</v>
       </c>
       <c r="B23" t="n">
         <v>1220</v>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C23" t="s">
+        <v>21</v>
       </c>
       <c r="D23" t="n">
         <v>5251</v>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>COMPANHIA DE GÁS DE MINAS GERAIS - GASMIG</t>
-        </is>
+      <c r="E23" t="s">
+        <v>52</v>
       </c>
       <c r="F23" t="n">
         <v>25</v>
@@ -2118,15 +2062,11 @@
       <c r="O23" t="n">
         <v>0</v>
       </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>MINAS GERAÇÃO DE VALOR</t>
-        </is>
-      </c>
-      <c r="Q23" t="inlineStr">
-        <is>
-          <t>GÁS COMPETITIVO- EXPANSÃO DA REDE DE GÁS NATURAL</t>
-        </is>
+      <c r="P23" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>53</v>
       </c>
       <c r="R23" t="n">
         <v>409881263</v>
@@ -2142,24 +2082,20 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" t="n">
         <v>2024</v>
       </c>
       <c r="B24" t="n">
         <v>1220</v>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C24" t="s">
+        <v>21</v>
       </c>
       <c r="D24" t="n">
         <v>5381</v>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
-        </is>
+      <c r="E24" t="s">
+        <v>54</v>
       </c>
       <c r="F24" t="n">
         <v>4</v>
@@ -2191,15 +2127,11 @@
       <c r="O24" t="n">
         <v>0</v>
       </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
-        </is>
+      <c r="P24" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>56</v>
       </c>
       <c r="R24" t="n">
         <v>4300000</v>
@@ -2215,24 +2147,20 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" t="n">
         <v>2024</v>
       </c>
       <c r="B25" t="n">
         <v>1220</v>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C25" t="s">
+        <v>21</v>
       </c>
       <c r="D25" t="n">
         <v>5381</v>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
-        </is>
+      <c r="E25" t="s">
+        <v>54</v>
       </c>
       <c r="F25" t="n">
         <v>4</v>
@@ -2264,15 +2192,11 @@
       <c r="O25" t="n">
         <v>0</v>
       </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
-        </is>
+      <c r="P25" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>56</v>
       </c>
       <c r="R25" t="n">
         <v>200000</v>
@@ -2288,24 +2212,20 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" t="n">
         <v>2024</v>
       </c>
       <c r="B26" t="n">
         <v>1220</v>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C26" t="s">
+        <v>21</v>
       </c>
       <c r="D26" t="n">
         <v>5381</v>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
-        </is>
+      <c r="E26" t="s">
+        <v>54</v>
       </c>
       <c r="F26" t="n">
         <v>4</v>
@@ -2337,15 +2257,11 @@
       <c r="O26" t="n">
         <v>0</v>
       </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
-        </is>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
-        </is>
+      <c r="P26" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>56</v>
       </c>
       <c r="R26" t="n">
         <v>1000</v>
@@ -2361,24 +2277,20 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" t="n">
         <v>2024</v>
       </c>
       <c r="B27" t="n">
         <v>1220</v>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C27" t="s">
+        <v>21</v>
       </c>
       <c r="D27" t="n">
         <v>5381</v>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>MINAS GERAIS ADMINISTRAÇÃO E SERVIÇOS S.A - MGS</t>
-        </is>
+      <c r="E27" t="s">
+        <v>54</v>
       </c>
       <c r="F27" t="n">
         <v>4</v>
@@ -2410,15 +2322,11 @@
       <c r="O27" t="n">
         <v>0</v>
       </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>SOLUÇÕES EM SERVIÇOS DE APOIO TÉCNICO-OPERACIONAL</t>
-        </is>
-      </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>INVESTIMENTOS EM ATIVO FIXO PARA PRESTAÇÃO DE SERVIÇO</t>
-        </is>
+      <c r="P27" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>56</v>
       </c>
       <c r="R27" t="n">
         <v>4000000</v>
@@ -2434,24 +2342,20 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" t="n">
         <v>2024</v>
       </c>
       <c r="B28" t="n">
         <v>1220</v>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C28" t="s">
+        <v>21</v>
       </c>
       <c r="D28" t="n">
         <v>5391</v>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
-        </is>
+      <c r="E28" t="s">
+        <v>57</v>
       </c>
       <c r="F28" t="n">
         <v>25</v>
@@ -2483,15 +2387,11 @@
       <c r="O28" t="n">
         <v>0</v>
       </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
-        </is>
-      </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>EXPANSÃO DO SISTEMA DE TRANSMISSÃO</t>
-        </is>
+      <c r="P28" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>59</v>
       </c>
       <c r="R28" t="n">
         <v>198940203</v>
@@ -2507,24 +2407,20 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" t="n">
         <v>2024</v>
       </c>
       <c r="B29" t="n">
         <v>1220</v>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C29" t="s">
+        <v>21</v>
       </c>
       <c r="D29" t="n">
         <v>5391</v>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
-        </is>
+      <c r="E29" t="s">
+        <v>57</v>
       </c>
       <c r="F29" t="n">
         <v>25</v>
@@ -2556,15 +2452,11 @@
       <c r="O29" t="n">
         <v>0</v>
       </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
-        </is>
-      </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>REFORMAS DE SUBESTAÇÕES E LINHAS DE TRANSMISSÃO</t>
-        </is>
+      <c r="P29" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>60</v>
       </c>
       <c r="R29" t="n">
         <v>241821909</v>
@@ -2580,24 +2472,20 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" t="n">
         <v>2024</v>
       </c>
       <c r="B30" t="n">
         <v>1220</v>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C30" t="s">
+        <v>21</v>
       </c>
       <c r="D30" t="n">
         <v>5391</v>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
-        </is>
+      <c r="E30" t="s">
+        <v>57</v>
       </c>
       <c r="F30" t="n">
         <v>25</v>
@@ -2629,15 +2517,11 @@
       <c r="O30" t="n">
         <v>0</v>
       </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>TRANSMISSÃO DE ENERGIA ELÉTRICA</t>
-        </is>
-      </c>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA TRANSMISSÃO</t>
-        </is>
+      <c r="P30" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>61</v>
       </c>
       <c r="R30" t="n">
         <v>30805275</v>
@@ -2653,24 +2537,20 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" t="n">
         <v>2024</v>
       </c>
       <c r="B31" t="n">
         <v>1220</v>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C31" t="s">
+        <v>21</v>
       </c>
       <c r="D31" t="n">
         <v>5391</v>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
-        </is>
+      <c r="E31" t="s">
+        <v>57</v>
       </c>
       <c r="F31" t="n">
         <v>25</v>
@@ -2702,15 +2582,11 @@
       <c r="O31" t="n">
         <v>0</v>
       </c>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
-        </is>
-      </c>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t>EXPANSÃO DO SISTEMA DE GERAÇÃO</t>
-        </is>
+      <c r="P31" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>63</v>
       </c>
       <c r="R31" t="n">
         <v>49096963</v>
@@ -2726,24 +2602,20 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" t="n">
         <v>2024</v>
       </c>
       <c r="B32" t="n">
         <v>1220</v>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C32" t="s">
+        <v>21</v>
       </c>
       <c r="D32" t="n">
         <v>5391</v>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
-        </is>
+      <c r="E32" t="s">
+        <v>57</v>
       </c>
       <c r="F32" t="n">
         <v>25</v>
@@ -2775,15 +2647,11 @@
       <c r="O32" t="n">
         <v>0</v>
       </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t>REFORMAS, MELHORIAS E AMPLIAÇÕES DE USINAS</t>
-        </is>
+      <c r="P32" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>64</v>
       </c>
       <c r="R32" t="n">
         <v>130600000</v>
@@ -2799,24 +2667,20 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" t="n">
         <v>2024</v>
       </c>
       <c r="B33" t="n">
         <v>1220</v>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C33" t="s">
+        <v>21</v>
       </c>
       <c r="D33" t="n">
         <v>5391</v>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
-        </is>
+      <c r="E33" t="s">
+        <v>57</v>
       </c>
       <c r="F33" t="n">
         <v>25</v>
@@ -2848,15 +2712,11 @@
       <c r="O33" t="n">
         <v>0</v>
       </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
-        </is>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA GERAÇÃO</t>
-        </is>
+      <c r="P33" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>65</v>
       </c>
       <c r="R33" t="n">
         <v>13194360</v>
@@ -2872,24 +2732,20 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" t="n">
         <v>2024</v>
       </c>
       <c r="B34" t="n">
         <v>1220</v>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C34" t="s">
+        <v>21</v>
       </c>
       <c r="D34" t="n">
         <v>5391</v>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>CEMIG GERAÇÃO E TRANSMISSÃO S.A - CEMIG GERAÇÃO E TRANSMISSÃO</t>
-        </is>
+      <c r="E34" t="s">
+        <v>57</v>
       </c>
       <c r="F34" t="n">
         <v>25</v>
@@ -2921,15 +2777,11 @@
       <c r="O34" t="n">
         <v>0</v>
       </c>
-      <c r="P34" t="inlineStr">
-        <is>
-          <t>GERAÇÃO DE ENERGIA ELÉTRICA</t>
-        </is>
-      </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t>INVESTIMENTOS EM PARTICIPAÇÕES SOCIETÁRIAS CEMIG GERAÇÃO E TRANSMISSÃO</t>
-        </is>
+      <c r="P34" t="s">
+        <v>62</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>66</v>
       </c>
       <c r="R34" t="n">
         <v>508846661</v>
@@ -2945,24 +2797,20 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" t="n">
         <v>2024</v>
       </c>
       <c r="B35" t="n">
         <v>1220</v>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C35" t="s">
+        <v>21</v>
       </c>
       <c r="D35" t="n">
         <v>5401</v>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
-        </is>
+      <c r="E35" t="s">
+        <v>67</v>
       </c>
       <c r="F35" t="n">
         <v>25</v>
@@ -2994,15 +2842,11 @@
       <c r="O35" t="n">
         <v>0</v>
       </c>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
-        </is>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t>EXECUÇÃO DO PLANO DE DESENVOLVIMENTO DA DISTRIBUIDORA (PDD)</t>
-        </is>
+      <c r="P35" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>69</v>
       </c>
       <c r="R35" t="n">
         <v>3487433034</v>
@@ -3018,24 +2862,20 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" t="n">
         <v>2024</v>
       </c>
       <c r="B36" t="n">
         <v>1220</v>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C36" t="s">
+        <v>21</v>
       </c>
       <c r="D36" t="n">
         <v>5401</v>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>CEMIG DISTRIBUIÇÃO S.A - CEMIG DISTRIBUIDORA</t>
-        </is>
+      <c r="E36" t="s">
+        <v>67</v>
       </c>
       <c r="F36" t="n">
         <v>25</v>
@@ -3067,15 +2907,11 @@
       <c r="O36" t="n">
         <v>0</v>
       </c>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t>DISTRIBUIÇÃO DE ENERGIA ELÉTRICA</t>
-        </is>
-      </c>
-      <c r="Q36" t="inlineStr">
-        <is>
-          <t>MANUTENÇÃO DA INFRAESTRUTURA DA DISTRIBUIÇÃO</t>
-        </is>
+      <c r="P36" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>70</v>
       </c>
       <c r="R36" t="n">
         <v>247223810</v>
@@ -3091,24 +2927,20 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" t="n">
         <v>2024</v>
       </c>
       <c r="B37" t="n">
         <v>1220</v>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C37" t="s">
+        <v>21</v>
       </c>
       <c r="D37" t="n">
         <v>5511</v>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
-        </is>
+      <c r="E37" t="s">
+        <v>71</v>
       </c>
       <c r="F37" t="n">
         <v>17</v>
@@ -3140,15 +2972,11 @@
       <c r="O37" t="n">
         <v>0</v>
       </c>
-      <c r="P37" t="inlineStr">
-        <is>
-          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
-        </is>
-      </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t>ADEQUAÇÃO DA INFRAESTRUTURA ADMINISTRATIVA E OPERACIONAL DA COPANOR</t>
-        </is>
+      <c r="P37" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>72</v>
       </c>
       <c r="R37" t="n">
         <v>2000000</v>
@@ -3164,24 +2992,20 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" t="n">
         <v>2024</v>
       </c>
       <c r="B38" t="n">
         <v>1220</v>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE DESENVOLVIMENTO ECONÔMICO - SEDE</t>
-        </is>
+      <c r="C38" t="s">
+        <v>21</v>
       </c>
       <c r="D38" t="n">
         <v>5511</v>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>COPASA - SERVIÇOS DE SANEAMENTO INTEGRADO DO NORTE E NORDESTE DE MINAS GERAIS S/A - COPANOR</t>
-        </is>
+      <c r="E38" t="s">
+        <v>71</v>
       </c>
       <c r="F38" t="n">
         <v>17</v>
@@ -3213,15 +3037,11 @@
       <c r="O38" t="n">
         <v>0</v>
       </c>
-      <c r="P38" t="inlineStr">
-        <is>
-          <t>SANEAMENTO E RESÍDUOS ESPECIAIS</t>
-        </is>
-      </c>
-      <c r="Q38" t="inlineStr">
-        <is>
-          <t>UNIVERSALIZAÇÃO DOS SERVIÇOS DE SANEAMENTO NA ÁREA DE ATUAÇÃO DA COPANOR</t>
-        </is>
+      <c r="P38" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>73</v>
       </c>
       <c r="R38" t="n">
         <v>45000000</v>
@@ -3237,24 +3057,20 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" t="n">
         <v>2024</v>
       </c>
       <c r="B39" t="n">
         <v>1300</v>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE INFRAESTRUTURA, MOBILIDADE E PARCERIA - SEINFRA</t>
-        </is>
+      <c r="C39" t="s">
+        <v>74</v>
       </c>
       <c r="D39" t="n">
         <v>5261</v>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>TREM METROPOLITANO DE BELO HORIZONTE S.A - TREM METROPOLITANO</t>
-        </is>
+      <c r="E39" t="s">
+        <v>75</v>
       </c>
       <c r="F39" t="n">
         <v>26</v>
@@ -3286,15 +3102,11 @@
       <c r="O39" t="n">
         <v>0</v>
       </c>
-      <c r="P39" t="inlineStr">
-        <is>
-          <t>APOIO ÀS POLÍTICAS PÚBLICAS</t>
-        </is>
-      </c>
-      <c r="Q39" t="inlineStr">
-        <is>
-          <t>MANUTENÇÃO E ADEQUAÇÃO DA INFRA-ESTRUTURA ADMINISTRATIVA E OPERACIONAL - TRANSPORTES METROPOLITANOS</t>
-        </is>
+      <c r="P39" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>76</v>
       </c>
       <c r="R39" t="n">
         <v>1000</v>
@@ -3310,24 +3122,20 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" t="n">
         <v>2024</v>
       </c>
       <c r="B40" t="n">
         <v>1500</v>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
-        </is>
+      <c r="C40" t="s">
+        <v>77</v>
       </c>
       <c r="D40" t="n">
         <v>5141</v>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
-        </is>
+      <c r="E40" t="s">
+        <v>78</v>
       </c>
       <c r="F40" t="n">
         <v>4</v>
@@ -3359,15 +3167,11 @@
       <c r="O40" t="n">
         <v>0</v>
       </c>
-      <c r="P40" t="inlineStr">
-        <is>
-          <t>SOLUÇÕES EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
-        </is>
-      </c>
-      <c r="Q40" t="inlineStr">
-        <is>
-          <t>MANUTENÇÃO DAS UNIDADES PREDIAIS</t>
-        </is>
+      <c r="P40" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>80</v>
       </c>
       <c r="R40" t="n">
         <v>3280000</v>
@@ -3383,24 +3187,20 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" t="n">
         <v>2024</v>
       </c>
       <c r="B41" t="n">
         <v>1500</v>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>SECRETARIA DE ESTADO DE PLANEJAMENTO E GESTÃO - SEPLAG</t>
-        </is>
+      <c r="C41" t="s">
+        <v>77</v>
       </c>
       <c r="D41" t="n">
         <v>5141</v>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>COMPANHIA DE TECNOLOGIA DA INFORMAÇÃO DO ESTADO DE MINAS GERAIS - PRODEMGE</t>
-        </is>
+      <c r="E41" t="s">
+        <v>78</v>
       </c>
       <c r="F41" t="n">
         <v>4</v>
@@ -3432,15 +3232,11 @@
       <c r="O41" t="n">
         <v>0</v>
       </c>
-      <c r="P41" t="inlineStr">
-        <is>
-          <t>SOLUÇÕES EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
-        </is>
-      </c>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>AQUISIÇÃO DE HARDWARES E SOFTWARES PARA PRESTAÇÃO DE SERVIÇOS EM TECNOLOGIA DA INFORMAÇÃO E COMUNICAÇÃO</t>
-        </is>
+      <c r="P41" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q41" t="s">
+        <v>81</v>
       </c>
       <c r="R41" t="n">
         <v>35386354</v>
@@ -3456,6 +3252,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
atualiza bancos 27/09 11:34
</commit_message>
<xml_diff>
--- a/bancos/SISOR/BASE_QDD_PLURIANUAL_INVEST.xlsx
+++ b/bancos/SISOR/BASE_QDD_PLURIANUAL_INVEST.xlsx
@@ -1021,16 +1021,16 @@
         </is>
       </c>
       <c r="R8" t="n">
-        <v>40000000</v>
+        <v>1062500000</v>
       </c>
       <c r="S8" t="n">
-        <v>40000000</v>
+        <v>1040500000</v>
       </c>
       <c r="T8" t="n">
-        <v>40000000</v>
+        <v>1040500000</v>
       </c>
       <c r="U8" t="n">
-        <v>40000000</v>
+        <v>1040500000</v>
       </c>
     </row>
     <row r="9">
@@ -1094,16 +1094,16 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>1062500000</v>
+        <v>40000000</v>
       </c>
       <c r="S9" t="n">
-        <v>1040500000</v>
+        <v>40000000</v>
       </c>
       <c r="T9" t="n">
-        <v>1040500000</v>
+        <v>40000000</v>
       </c>
       <c r="U9" t="n">
-        <v>1040500000</v>
+        <v>40000000</v>
       </c>
     </row>
     <row r="10">
@@ -1167,16 +1167,16 @@
         </is>
       </c>
       <c r="R10" t="n">
-        <v>100000000</v>
+        <v>97500000</v>
       </c>
       <c r="S10" t="n">
-        <v>100000000</v>
+        <v>97500000</v>
       </c>
       <c r="T10" t="n">
-        <v>100000000</v>
+        <v>97500000</v>
       </c>
       <c r="U10" t="n">
-        <v>100000000</v>
+        <v>97500000</v>
       </c>
     </row>
     <row r="11">
@@ -1240,16 +1240,16 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>97500000</v>
+        <v>100000000</v>
       </c>
       <c r="S11" t="n">
-        <v>97500000</v>
+        <v>100000000</v>
       </c>
       <c r="T11" t="n">
-        <v>97500000</v>
+        <v>100000000</v>
       </c>
       <c r="U11" t="n">
-        <v>97500000</v>
+        <v>100000000</v>
       </c>
     </row>
     <row r="12">
@@ -3214,13 +3214,13 @@
         <v>1000</v>
       </c>
       <c r="S38" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="T38" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="U38" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="39">

</xml_diff>